<commit_message>
Correct physician anesthesia DOP ages for core and pediatric privileges
Replace adult 18+ / pediatric 2 months–17 years with core privileges for patients 2 years and older and pediatric privileges for patients 2 months and older, which still require a pediatric anesthesiology fellowship and PALS.

Co-authored-by: gorin-research-repo <gorin-research-repo@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/case-logs/ANESTHESIA_(PHYSICIAN)_CASE_LOG_TEMPLATE_July_8_2026.xlsx
+++ b/case-logs/ANESTHESIA_(PHYSICIAN)_CASE_LOG_TEMPLATE_July_8_2026.xlsx
@@ -15,11 +15,11 @@
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
     <sheet name="Applicant Information" sheetId="2" r:id="rId2"/>
-    <sheet name="Adult Anesthesia" sheetId="3" r:id="rId3"/>
-    <sheet name="Pediatric Anesthesia" sheetId="4" r:id="rId4"/>
+    <sheet name="Core (2 years and older)" sheetId="3" r:id="rId3"/>
+    <sheet name="Pediatric (2 months and older)" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Adult Anesthesia'!$B$1:$H$1644</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Core (2 years and older)'!$B$1:$H$1644</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -474,7 +474,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Complete the appropriate sections (tabs) of the workbook corresponding to the privilege categories being requested (e.g., Adult Anesthesia, Pediatric Anesthesia).</a:t>
+            <a:t>Complete the appropriate sections (tabs) of the workbook corresponding to the privilege categories being requested (e.g., Core (2 years and older), Pediatric (2 months and older)).</a:t>
           </a:r>
         </a:p>
         <a:p>

</xml_diff>

<commit_message>
Restructure physician anesthesia DOP into core age bands plus 2 months–2 years
Keep one core section for patients 2 years and older, with grantable bands of 2–12, 13–17, and 18+. Move fellowship and PALS into a separate 2 months–2 years section and note that those extra requirements apply only to that age group.

Co-authored-by: gorin-research-repo <gorin-research-repo@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/case-logs/ANESTHESIA_(PHYSICIAN)_CASE_LOG_TEMPLATE_July_8_2026.xlsx
+++ b/case-logs/ANESTHESIA_(PHYSICIAN)_CASE_LOG_TEMPLATE_July_8_2026.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
     <sheet name="Applicant Information" sheetId="2" r:id="rId2"/>
     <sheet name="Core (2 years and older)" sheetId="3" r:id="rId3"/>
-    <sheet name="Pediatric (2 months and older)" sheetId="4" r:id="rId4"/>
+    <sheet name="Pediatric (2 months to 2 years)" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Core (2 years and older)'!$B$1:$H$1644</definedName>
@@ -474,7 +474,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Complete the appropriate sections (tabs) of the workbook corresponding to the privilege categories being requested (e.g., Core (2 years and older), Pediatric (2 months and older)).</a:t>
+            <a:t>Complete the appropriate sections (tabs) of the workbook corresponding to the privilege categories being requested (e.g., Core (2 years and older), Pediatric (2 months to 2 years)).</a:t>
           </a:r>
         </a:p>
         <a:p>

</xml_diff>

<commit_message>
Use one Anesthesiology grid with 2-months+ and any-age privilege lines
Remove the second pediatric section. Request age on the same grid: patients 2 months of age and older, or patients of any age, with pediatric anesthesiology certification and PALS listed under the any-age line.

Co-authored-by: gorin-research-repo <gorin-research-repo@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/case-logs/ANESTHESIA_(PHYSICIAN)_CASE_LOG_TEMPLATE_July_8_2026.xlsx
+++ b/case-logs/ANESTHESIA_(PHYSICIAN)_CASE_LOG_TEMPLATE_July_8_2026.xlsx
@@ -15,11 +15,11 @@
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
     <sheet name="Applicant Information" sheetId="2" r:id="rId2"/>
-    <sheet name="Core (2 years and older)" sheetId="3" r:id="rId3"/>
-    <sheet name="Pediatric (2 months to 2 years)" sheetId="4" r:id="rId4"/>
+    <sheet name="2 months and older" sheetId="3" r:id="rId3"/>
+    <sheet name="Any age" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Core (2 years and older)'!$B$1:$H$1644</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 months and older'!$B$1:$H$1644</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -474,7 +474,7 @@
               <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Complete the appropriate sections (tabs) of the workbook corresponding to the privilege categories being requested (e.g., Core (2 years and older), Pediatric (2 months to 2 years)).</a:t>
+            <a:t>Complete the appropriate sections (tabs) of the workbook corresponding to the privilege categories being requested (e.g., 2 months and older, Any age).</a:t>
           </a:r>
         </a:p>
         <a:p>

</xml_diff>